<commit_message>
TD3: line chart, no frozen header
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NXi9t7is4XGBcVStY3YFum
</commit_message>
<xml_diff>
--- a/TD3_mix_energetique.xlsx
+++ b/TD3_mix_energetique.xlsx
@@ -182,7 +182,7 @@
             </a:pPr>
             <a:r>
               <a:rPr sz="1200" b="0"/>
-              <a:t>Production par filière (MW). Au-dessus de la courbe rouge : vente. Négatif : charge des stockages.</a:t>
+              <a:t>Production par filière et demande (MW)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -190,236 +190,18 @@
       <overlay val="0"/>
     </title>
     <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="stacked"/>
+      <lineChart>
+        <grouping val="standard"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'TD3'!F3</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="F2B701"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="F2B701"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'TD3'!$A$4:$A$27</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'TD3'!$F$4:$F$27</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'TD3'!G3</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="1F77B4"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="1F77B4"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'TD3'!$A$4:$A$27</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'TD3'!$G$4:$G$27</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <strRef>
-              <f>'TD3'!D3</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="FFE34D"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="FFE34D"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'TD3'!$A$4:$A$27</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'TD3'!$D$4:$D$27</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <tx>
-            <strRef>
-              <f>'TD3'!E3</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="7CC47F"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="7CC47F"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'TD3'!$A$4:$A$27</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'TD3'!$E$4:$E$27</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="4"/>
-          <order val="4"/>
-          <tx>
-            <strRef>
-              <f>'TD3'!I3</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="9467BD"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="9467BD"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'TD3'!$A$4:$A$27</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'TD3'!$I$4:$I$27</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="5"/>
-          <order val="5"/>
-          <tx>
-            <strRef>
-              <f>'TD3'!K3</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="17BECF"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="17BECF"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'TD3'!$A$4:$A$27</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'TD3'!$K$4:$K$27</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="6"/>
-          <order val="6"/>
-          <tx>
-            <strRef>
-              <f>'TD3'!M3</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="A0A0A0"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:solidFill>
-                <a:srgbClr val="A0A0A0"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'TD3'!$A$4:$A$27</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'TD3'!$M$4:$M$27</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="30"/>
-        <overlap val="100"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="7"/>
-          <order val="7"/>
           <tx>
             <strRef>
               <f>'TD3'!B3</f>
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="38000">
               <a:solidFill>
                 <a:srgbClr val="D62728"/>
               </a:solidFill>
@@ -434,9 +216,230 @@
               </a:ln>
             </spPr>
           </marker>
+          <cat>
+            <numRef>
+              <f>'TD3'!$A$4:$A$27</f>
+            </numRef>
+          </cat>
           <val>
             <numRef>
               <f>'TD3'!$B$4:$B$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'TD3'!F3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
+              <a:solidFill>
+                <a:srgbClr val="FF7F0E"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'TD3'!$A$4:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'TD3'!$F$4:$F$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'TD3'!G3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
+              <a:solidFill>
+                <a:srgbClr val="1F77B4"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'TD3'!$A$4:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'TD3'!$G$4:$G$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'TD3'!D3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
+              <a:solidFill>
+                <a:srgbClr val="E6B800"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'TD3'!$A$4:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'TD3'!$D$4:$D$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'TD3'!E3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
+              <a:solidFill>
+                <a:srgbClr val="2CA02C"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'TD3'!$A$4:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'TD3'!$E$4:$E$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <strRef>
+              <f>'TD3'!I3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
+              <a:solidFill>
+                <a:srgbClr val="9467BD"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'TD3'!$A$4:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'TD3'!$I$4:$I$27</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <tx>
+            <strRef>
+              <f>'TD3'!K3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
+              <a:solidFill>
+                <a:srgbClr val="17BECF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'TD3'!$A$4:$A$27</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'TD3'!$K$4:$K$27</f>
             </numRef>
           </val>
           <smooth val="0"/>

</xml_diff>